<commit_message>
Renamed nuclear reloading to refuelling and shifted example demand.
Co-authored-by: YuriBae0106 <106811326+YuriBae0106@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/tech_data.xlsx
+++ b/data/tech_data.xlsx
@@ -1040,7 +1040,7 @@
     <row r="36" ht="15" customHeight="1" s="8">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>reload_duration</t>
+          <t>refuel_duration</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -1050,12 +1050,12 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>duration of planned reload shutdown</t>
+          <t>duration of planned refuelling shutdown</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Used in makenuclear; set 0 to disable reload downtime.</t>
+          <t>Used in makenuclear; set 0 to disable refuelling downtime.</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1320,7 @@
     <row r="51" ht="15" customHeight="1" s="8">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>reload_fraction_per_year</t>
+          <t>refuel_fraction_per_year</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -1330,7 +1330,7 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>minimum planned reload requirement per unit-year</t>
+          <t>minimum planned refuelling requirement per unit-year</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -1898,7 +1898,7 @@
     <row r="19" ht="15" customHeight="1" s="8">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>reload_duration</t>
+          <t>refuel_duration</t>
         </is>
       </c>
       <c r="B19" s="7" t="n">
@@ -1994,7 +1994,7 @@
     <row r="25" ht="15" customHeight="1" s="8">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>reload_fraction_per_year</t>
+          <t>refuel_fraction_per_year</t>
         </is>
       </c>
       <c r="B25" s="7" t="n">

</xml_diff>